<commit_message>
Initial hMSM code release
</commit_message>
<xml_diff>
--- a/eval/Final_Results.xlsx
+++ b/eval/Final_Results.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\FinalTop\eval\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\top_optim\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C94092A-4D4E-4EFD-A51A-96F9A0D8E433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3368DF4-5068-46AA-BB0A-D5AE868C53F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DC97868F-0C32-49C4-BD1D-CDEEAEA189B3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3A7F9FB1-002B-410C-B375-D447C91048F8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Wheel_Gripper_Comparison" sheetId="1" r:id="rId1"/>
-    <sheet name="Beam_Comparison" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,19 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="22">
-  <si>
-    <t>G model</t>
-  </si>
-  <si>
-    <t>NH1</t>
-  </si>
-  <si>
-    <t>NH2</t>
-  </si>
-  <si>
-    <t>StVK</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="22">
   <si>
     <t>Default</t>
   </si>
@@ -66,15 +53,6 @@
     <t>Kerner</t>
   </si>
   <si>
-    <t>Wheel</t>
-  </si>
-  <si>
-    <t>Gripper</t>
-  </si>
-  <si>
-    <t>Micro</t>
-  </si>
-  <si>
     <t>Small</t>
   </si>
   <si>
@@ -84,7 +62,34 @@
     <t>Large</t>
   </si>
   <si>
-    <t>Relative Difference from Default</t>
+    <t>Load Case</t>
+  </si>
+  <si>
+    <t>LP</t>
+  </si>
+  <si>
+    <t>LPA</t>
+  </si>
+  <si>
+    <t>NH2 Constant</t>
+  </si>
+  <si>
+    <t>Tip</t>
+  </si>
+  <si>
+    <t>Gripper</t>
+  </si>
+  <si>
+    <t>NH1</t>
+  </si>
+  <si>
+    <t>NH2</t>
+  </si>
+  <si>
+    <t>Wheel</t>
+  </si>
+  <si>
+    <t>Geometry</t>
   </si>
   <si>
     <t>Where:</t>
@@ -93,30 +98,23 @@
     <t xml:space="preserve">% Diff = abs( (Ug-Ud)/Ud) </t>
   </si>
   <si>
-    <t>Load Magnitude</t>
+    <t>Relative Difference from Default (NH2)</t>
   </si>
   <si>
-    <t>Magnetized Tip</t>
+    <t>Hill</t>
   </si>
   <si>
-    <t>Load Case</t>
-  </si>
-  <si>
-    <t>Beam Comparison with NH2 Constant</t>
-  </si>
-  <si>
-    <t>Geometry</t>
+    <t>SVK</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +133,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -161,199 +165,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="170" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -400,8 +221,15 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Model Affect on Wheel Displacement</a:t>
+              <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Model effect on gripper displacement</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -447,11 +275,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$B$2</c:f>
+              <c:f>Sheet1!$B$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NH1</c:v>
+                  <c:v>SVK</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -468,9 +296,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$3:$A$6</c:f>
+              <c:f>Sheet1!$A$20:$A$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -481,35 +309,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$B$3:$B$6</c:f>
+              <c:f>Sheet1!$B$20:$B$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>9.5284951539999998</c:v>
+                  <c:v>9.8244659297066494</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9729490089999997</c:v>
+                  <c:v>7.1216328725202001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.53033866</c:v>
+                  <c:v>6.6593933989619503</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.986455479</c:v>
+                  <c:v>6.2782669680430798</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.17196340201785</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.7303847693785599</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.5034105576629297</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BBB9-45DC-9AD6-FEEC0DA39DC3}"/>
+              <c16:uniqueId val="{00000000-77B7-4AA5-AB12-3649633E73A0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -518,11 +364,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$C$2</c:f>
+              <c:f>Sheet1!$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NH2</c:v>
+                  <c:v>NH1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -539,9 +385,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$3:$A$6</c:f>
+              <c:f>Sheet1!$A$20:$A$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -552,35 +398,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$C$3:$C$6</c:f>
+              <c:f>Sheet1!$C$20:$C$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>9.5289460140000006</c:v>
+                  <c:v>9.7224180529970603</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9738571880000002</c:v>
+                  <c:v>7.1373449227254699</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.5313767699999996</c:v>
+                  <c:v>6.6838920896256004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.9871286640000001</c:v>
+                  <c:v>6.3077024160821704</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.1558525860663007</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.7296829173204999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.5094799929563196</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-BBB9-45DC-9AD6-FEEC0DA39DC3}"/>
+              <c16:uniqueId val="{00000000-4543-495D-B1F0-FCF9CCF7A5B4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -589,11 +453,11 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$D$2</c:f>
+              <c:f>Sheet1!$D$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>StVK</c:v>
+                  <c:v>NH2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -610,9 +474,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$3:$A$6</c:f>
+              <c:f>Sheet1!$A$20:$A$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -623,35 +487,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$D$3:$D$6</c:f>
+              <c:f>Sheet1!$D$20:$D$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>9.6586474239999998</c:v>
+                  <c:v>9.7234960825768297</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9651783140000001</c:v>
+                  <c:v>7.13992117567118</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.5110522409999998</c:v>
+                  <c:v>6.6868031512495696</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>8.0195223710000008</c:v>
+                  <c:v>6.3109014900087397</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.1577491532673392</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.7318502195569998</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.5117951079559404</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-BBB9-45DC-9AD6-FEEC0DA39DC3}"/>
+              <c16:uniqueId val="{00000001-4543-495D-B1F0-FCF9CCF7A5B4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -665,11 +547,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="594455520"/>
-        <c:axId val="594456000"/>
+        <c:axId val="2010574927"/>
+        <c:axId val="391670767"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="594455520"/>
+        <c:axId val="2010574927"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -695,10 +577,16 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
-                  <a:t>Shear Modulus Relation</a:t>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Shear modulus relation</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -753,7 +641,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -768,7 +656,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="594456000"/>
+        <c:crossAx val="391670767"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -776,7 +664,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="594456000"/>
+        <c:axId val="391670767"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -802,13 +690,27 @@
               <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
-                <a:pPr>
+                <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                  <a:lnSpc>
+                    <a:spcPct val="100000"/>
+                  </a:lnSpc>
+                  <a:spcBef>
+                    <a:spcPts val="0"/>
+                  </a:spcBef>
+                  <a:spcAft>
+                    <a:spcPts val="0"/>
+                  </a:spcAft>
+                  <a:buClrTx/>
+                  <a:buSzTx/>
+                  <a:buFontTx/>
+                  <a:buNone/>
+                  <a:tabLst/>
                   <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="tx1">
+                      <a:sysClr val="windowText" lastClr="000000">
                         <a:lumMod val="65000"/>
                         <a:lumOff val="35000"/>
-                      </a:schemeClr>
+                      </a:sysClr>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -816,13 +718,27 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
-                  <a:t>Average Displacement Magnitude</a:t>
+                  <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Average displacement measure, Qₘ (mm)</a:t>
                 </a:r>
-                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="2.2341607131194711E-2"/>
+              <c:y val="0.14953832613770085"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -835,13 +751,27 @@
             <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
-              <a:pPr>
+              <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+                <a:lnSpc>
+                  <a:spcPct val="100000"/>
+                </a:lnSpc>
+                <a:spcBef>
+                  <a:spcPts val="0"/>
+                </a:spcBef>
+                <a:spcAft>
+                  <a:spcPts val="0"/>
+                </a:spcAft>
+                <a:buClrTx/>
+                <a:buSzTx/>
+                <a:buFontTx/>
+                <a:buNone/>
+                <a:tabLst/>
                 <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="tx1">
+                    <a:sysClr val="windowText" lastClr="000000">
                       <a:lumMod val="65000"/>
                       <a:lumOff val="35000"/>
-                    </a:schemeClr>
+                    </a:sysClr>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -852,7 +782,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -883,7 +813,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="594455520"/>
+        <c:crossAx val="2010574927"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1004,15 +934,16 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:sysClr>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>Model Affect on Gripper Displacement</a:t>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Model effect</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" baseline="0"/>
+              <a:t> on w</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>heel displacement</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1058,11 +989,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$B$9</c:f>
+              <c:f>Sheet1!$G$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NH1</c:v>
+                  <c:v>SVK</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1079,9 +1010,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$10:$A$13</c:f>
+              <c:f>Sheet1!$F$20:$F$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -1092,35 +1023,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$B$10:$B$13</c:f>
+              <c:f>Sheet1!$G$20:$G$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>18.421462741213698</c:v>
+                  <c:v>18.999836109635002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.266254811593701</c:v>
+                  <c:v>17.9942031022752</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17.154739436798899</c:v>
+                  <c:v>17.898851255607799</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.596416562498199</c:v>
+                  <c:v>17.828724632559101</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18.273403916763399</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.144490048353099</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18.0848329565383</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2272-4359-AC1C-A354B97A2524}"/>
+              <c16:uniqueId val="{00000000-A84E-418F-9027-C997ED6BAEF6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1129,11 +1078,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$C$9</c:f>
+              <c:f>Sheet1!$H$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NH2</c:v>
+                  <c:v>NH1</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1150,9 +1099,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$10:$A$13</c:f>
+              <c:f>Sheet1!$F$20:$F$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -1163,35 +1112,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$C$10:$C$13</c:f>
+              <c:f>Sheet1!$H$20:$H$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>18.416951952933001</c:v>
+                  <c:v>18.960935417712399</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.267316870122901</c:v>
+                  <c:v>17.929346810569498</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17.157242310400498</c:v>
+                  <c:v>17.829620432322201</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.5947611027206</c:v>
+                  <c:v>17.755691809499801</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18.218137121061599</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.085211123354199</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18.023485724756899</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2272-4359-AC1C-A354B97A2524}"/>
+              <c16:uniqueId val="{00000001-A84E-418F-9027-C997ED6BAEF6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1200,11 +1167,11 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$D$9</c:f>
+              <c:f>Sheet1!$I$19</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>StVK</c:v>
+                  <c:v>NH2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1221,9 +1188,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Wheel_Gripper_Comparison!$A$10:$A$13</c:f>
+              <c:f>Sheet1!$F$20:$F$26</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
                   <c:v>Default</c:v>
                 </c:pt>
@@ -1234,35 +1201,53 @@
                   <c:v>Mooney</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>Hill</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>Kerner</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>LP</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>LPA</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Wheel_Gripper_Comparison!$D$10:$D$13</c:f>
+              <c:f>Sheet1!$I$20:$I$26</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>18.475893918431499</c:v>
+                  <c:v>18.953478159908499</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17.345315007912301</c:v>
+                  <c:v>17.933775911685199</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>17.237104830960799</c:v>
+                  <c:v>17.837091601035802</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.667195454988001</c:v>
+                  <c:v>17.765996232382701</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18.216916221474101</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>18.086176589070998</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18.025678930195902</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-2272-4359-AC1C-A354B97A2524}"/>
+              <c16:uniqueId val="{00000002-A84E-418F-9027-C997ED6BAEF6}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1276,11 +1261,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="750065152"/>
-        <c:axId val="750081472"/>
+        <c:axId val="635417007"/>
+        <c:axId val="391661647"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="750065152"/>
+        <c:axId val="635417007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1314,7 +1299,7 @@
                       </a:sysClr>
                     </a:solidFill>
                   </a:rPr>
-                  <a:t>Shear Modulus Relation</a:t>
+                  <a:t>Shear modulus relation</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1370,7 +1355,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1385,7 +1370,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="750081472"/>
+        <c:crossAx val="391661647"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1393,7 +1378,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="750081472"/>
+        <c:axId val="391661647"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1441,11 +1426,19 @@
                       </a:sysClr>
                     </a:solidFill>
                   </a:rPr>
-                  <a:t>Average Displacement Magnitude</a:t>
+                  <a:t>Average displacement measure, Qₘ (mm)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="1.9570195362942373E-2"/>
+              <c:y val="0.15414949299546585"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -1475,7 +1468,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1506,7 +1499,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="750065152"/>
+        <c:crossAx val="635417007"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1627,8 +1620,8 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Model Affect on Beam Loading</a:t>
+              <a:rPr lang="en-US" sz="1100"/>
+              <a:t>Model effect on beam displacement</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1674,7 +1667,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Beam_Comparison!$B$2</c:f>
+              <c:f>Sheet1!$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1695,54 +1688,48 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Beam_Comparison!$A$3:$A$7</c:f>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Micro</c:v>
+                  <c:v>Small</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Small</c:v>
+                  <c:v>Medium</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Medium</c:v>
+                  <c:v>Large</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Large</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Magnetized Tip</c:v>
+                  <c:v>Tip</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Beam_Comparison!$B$3:$B$7</c:f>
+              <c:f>Sheet1!$B$3:$B$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.3491828990000001</c:v>
+                  <c:v>1.3895611944545101</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.5914016670000004</c:v>
+                  <c:v>4.70931514688424</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.0140517329999996</c:v>
+                  <c:v>9.3909205349798395</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.2493070320000008</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.3528580320000003</c:v>
+                  <c:v>4.4203874392245099</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3898-4C37-9E1D-F5C77775023A}"/>
+              <c16:uniqueId val="{00000000-AA15-4D64-9281-AB08C4F0A76D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1751,7 +1738,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Beam_Comparison!$C$2</c:f>
+              <c:f>Sheet1!$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1772,54 +1759,48 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Beam_Comparison!$A$3:$A$7</c:f>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Micro</c:v>
+                  <c:v>Small</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Small</c:v>
+                  <c:v>Medium</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Medium</c:v>
+                  <c:v>Large</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Large</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Magnetized Tip</c:v>
+                  <c:v>Tip</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Beam_Comparison!$C$3:$C$7</c:f>
+              <c:f>Sheet1!$C$3:$C$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.47367235699999999</c:v>
+                  <c:v>0.48453066402455303</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.848991979</c:v>
+                  <c:v>1.89002910510055</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.45726975</c:v>
+                  <c:v>5.8561611945997702</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.7607147589999999</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.3642715169999997</c:v>
+                  <c:v>4.4381703570595796</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3898-4C37-9E1D-F5C77775023A}"/>
+              <c16:uniqueId val="{00000001-AA15-4D64-9281-AB08C4F0A76D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1828,7 +1809,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Beam_Comparison!$D$2</c:f>
+              <c:f>Sheet1!$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1849,54 +1830,48 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Beam_Comparison!$A$3:$A$7</c:f>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Micro</c:v>
+                  <c:v>Small</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Small</c:v>
+                  <c:v>Medium</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Medium</c:v>
+                  <c:v>Large</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Large</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Magnetized Tip</c:v>
+                  <c:v>Tip</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Beam_Comparison!$D$3:$D$7</c:f>
+              <c:f>Sheet1!$D$3:$D$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.40781563900000001</c:v>
+                  <c:v>0.41685443010163098</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.6018056789999999</c:v>
+                  <c:v>1.6364320804784001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.0412965669999998</c:v>
+                  <c:v>5.31695784908832</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.229179222</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.3652269190000004</c:v>
+                  <c:v>4.43961470353669</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-3898-4C37-9E1D-F5C77775023A}"/>
+              <c16:uniqueId val="{00000002-AA15-4D64-9281-AB08C4F0A76D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1905,11 +1880,11 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Beam_Comparison!$E$2</c:f>
+              <c:f>Sheet1!$E$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Kerner</c:v>
+                  <c:v>Hill</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1926,54 +1901,263 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Beam_Comparison!$A$3:$A$7</c:f>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Micro</c:v>
+                  <c:v>Small</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Small</c:v>
+                  <c:v>Medium</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Medium</c:v>
+                  <c:v>Large</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Large</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Magnetized Tip</c:v>
+                  <c:v>Tip</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Beam_Comparison!$E$3:$E$7</c:f>
+              <c:f>Sheet1!$E$3:$E$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.68377695299999997</c:v>
+                  <c:v>0.36905398128043698</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.6036390140000001</c:v>
+                  <c:v>1.45456229910751</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.6174345839999997</c:v>
+                  <c:v>4.88857483724105</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7.0634611239999998</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.361258791</c:v>
+                  <c:v>4.4406803791778398</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-3898-4C37-9E1D-F5C77775023A}"/>
+              <c16:uniqueId val="{00000003-AA15-4D64-9281-AB08C4F0A76D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Kerner</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Small</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Medium</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Large</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Tip</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$F$3:$F$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.69650778599999996</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6499463840000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.154769494</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.4336164349900598</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-AA15-4D64-9281-AB08C4F0A76D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>LP</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Small</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Medium</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Large</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Tip</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$3:$G$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.59520169406391599</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.2937069970340298</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.5969477717673701</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.4357324774038096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-AA15-4D64-9281-AB08C4F0A76D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>LPA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$3:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Small</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Medium</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Large</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Tip</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$H$3:$H$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.55056005375619499</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.13261506819175</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.3168236910215301</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.4367143228592703</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-AA15-4D64-9281-AB08C4F0A76D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1987,11 +2171,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="750108832"/>
-        <c:axId val="750109792"/>
+        <c:axId val="2038401952"/>
+        <c:axId val="1651114896"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="750108832"/>
+        <c:axId val="2038401952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2018,7 +2202,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>Beam Load Case</a:t>
+                  <a:t>Load case</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -2074,7 +2258,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -2089,7 +2273,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="750109792"/>
+        <c:crossAx val="1651114896"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2097,7 +2281,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="750109792"/>
+        <c:axId val="1651114896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2145,7 +2329,7 @@
                       </a:sysClr>
                     </a:solidFill>
                   </a:rPr>
-                  <a:t>Average Displacement Magnitude</a:t>
+                  <a:t>Average Free-End Displacement Magnitude, Qₘ (mm)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -2179,7 +2363,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2210,7 +2394,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="750108832"/>
+        <c:crossAx val="2038401952"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2224,6 +2408,29 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="1"/>
+        <c:txPr>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+      </c:legendEntry>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -3930,23 +4137,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>605118</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>386081</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>169757</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>168086</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>119530</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>77047</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>169757</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FAF1678-048B-99B1-5FFA-4A7DADBE3E17}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D42AF93-5596-AB77-AEA1-DA9AD1EBC6D7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3966,23 +4173,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>605118</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>421640</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>85090</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>179294</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>89647</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>116841</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>85090</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
+        <xdr:cNvPr id="4" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C12985BF-C736-6E55-C16B-BD73B67BC148}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{77E7D27D-0D3B-530E-64D5-B895DF969252}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4000,30 +4207,25 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>3810</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>10991</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>5862</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>326048</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:rowOff>1466</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A797E3E9-AF31-FAFC-1992-18F75FFCB194}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6782E8AA-3DEB-43C2-1E2D-3CA12C52A7DE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4035,91 +4237,166 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>268077</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>52329</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="224229" cy="173766"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="TextBox 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEB7D51B-9DDC-F3B0-A3CC-A919500A8097}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8181860" y="9967510"/>
+              <a:ext cx="224229" cy="173766"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSub>
+                      <m:sSubPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSubPr>
+                      <m:e>
+                        <m:r>
+                          <m:rPr>
+                            <m:sty m:val="p"/>
+                          </m:rPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>Q</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sub>
+                        <m:r>
+                          <m:rPr>
+                            <m:sty m:val="p"/>
+                          </m:rPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>m</m:t>
+                        </m:r>
+                      </m:sub>
+                    </m:sSub>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="TextBox 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEB7D51B-9DDC-F3B0-A3CC-A919500A8097}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8181860" y="9967510"/>
+              <a:ext cx="224229" cy="173766"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>Q_m</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1100"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FCA44438-3D2B-49C3-AEC5-368563795A38}" name="Table3" displayName="Table3" ref="A2:D6" totalsRowShown="0">
-  <autoFilter ref="A2:D6" xr:uid="{FCA44438-3D2B-49C3-AEC5-368563795A38}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{10BE39A2-D58C-4415-B31A-E7D54B6146B7}" name="G model"/>
-    <tableColumn id="2" xr3:uid="{82D8A7D9-165E-49C3-9BBA-5C7CCF4E0B90}" name="NH1" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{6FA4CC7A-F19D-4051-8004-C8A708C3ABF0}" name="NH2" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{34A0C971-0CE5-4343-A781-B6485D9A649A}" name="StVK" dataDxfId="3"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F98B1F19-8AAE-4F39-9AE7-0F32C71F1F3F}" name="Table4" displayName="Table4" ref="A9:D13" totalsRowShown="0">
-  <autoFilter ref="A9:D13" xr:uid="{F98B1F19-8AAE-4F39-9AE7-0F32C71F1F3F}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{72E8BBB5-8A10-4EFF-B75B-A9B4347ABF4C}" name="G model"/>
-    <tableColumn id="2" xr3:uid="{C4C5C7A6-8547-4AA4-B067-90B7D8E52B95}" name="NH1" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{8A9876E2-2BE6-4BFE-9FE6-00BCC5A4596A}" name="NH2" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{D52BB815-B6A5-494E-B26C-07E95A6CF888}" name="StVK" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4839363F-B9B0-4E99-BC21-6BC51B855E48}" name="Table5" displayName="Table5" ref="A17:D19" totalsRowShown="0" dataDxfId="17" dataCellStyle="Percent">
-  <autoFilter ref="A17:D19" xr:uid="{4839363F-B9B0-4E99-BC21-6BC51B855E48}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{B47D74DD-FA03-4401-964F-485ABBC8E85E}" name="Geometry"/>
-    <tableColumn id="2" xr3:uid="{BF908CE0-ED53-49DD-A803-878A9E9653F4}" name="Guth" dataDxfId="16" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((C10-C9)/C9)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{AF3E19AD-0890-4D34-BDED-1E7928398A92}" name="Mooney" dataDxfId="15" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((C11-C9)/C9)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC2B6ECF-0580-4856-8BBB-9CF67ABFE4F0}" name="Kerner" dataDxfId="14" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((C12-C9)/C9)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}" name="Table1" displayName="Table1" ref="A11:D16" totalsRowShown="0" dataDxfId="13" dataCellStyle="Percent">
-  <autoFilter ref="A11:D16" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1C96DD68-5388-41C8-80A4-631AF2530025}" name="Load Case"/>
-    <tableColumn id="2" xr3:uid="{C0C49FD7-8D17-437F-88C8-BB6258B99219}" name="Guth" dataDxfId="12" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((C3-B3)/B3)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{CB5631BD-80FB-4B0B-BC78-3E45F11C5622}" name="Mooney" dataDxfId="11" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((D3-B3)/B3)</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{64489D84-8154-4AB7-B213-01F3A56C4E26}" name="Kerner" dataDxfId="10" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS((E3-B3)/B3)</calculatedColumnFormula>
-    </tableColumn>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1636F957-79EA-4A9C-A088-0551A65C1F5C}" name="Table2" displayName="Table2" ref="A2:E7" totalsRowShown="0">
-  <autoFilter ref="A2:E7" xr:uid="{1636F957-79EA-4A9C-A088-0551A65C1F5C}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{BBB9A9AD-3816-4FCF-910B-BC91E45978F8}" name="Load Magnitude"/>
-    <tableColumn id="2" xr3:uid="{C2C97874-87BF-4F49-8E77-46CBD4B4BE4A}" name="Default" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{2269703A-CD27-4542-B024-242B1A805057}" name="Guth" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{CF64BBBD-0D58-4197-9737-466E1D604376}" name="Mooney" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{2F62C0DF-5422-48A6-88EC-800D14AC8CAF}" name="Kerner" dataDxfId="6"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4438,99 +4715,161 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDFE2C64-06DF-4408-84BC-5CD53FB648D2}">
-  <dimension ref="A1:D21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FE9910B-14B0-45DF-9EF7-8E53608CE1DC}">
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="10.77734375" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" t="s">
         <v>8</v>
       </c>
+      <c r="H2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
-        <v>9.5284951539999998</v>
-      </c>
-      <c r="C3" s="4">
-        <v>9.5289460140000006</v>
-      </c>
-      <c r="D3" s="4">
-        <v>9.6586474239999998</v>
+      <c r="B3">
+        <v>1.3895611944545101</v>
+      </c>
+      <c r="C3">
+        <v>0.48453066402455303</v>
+      </c>
+      <c r="D3">
+        <v>0.41685443010163098</v>
+      </c>
+      <c r="E3">
+        <v>0.36905398128043698</v>
+      </c>
+      <c r="F3">
+        <v>0.69650778599999996</v>
+      </c>
+      <c r="G3">
+        <v>0.59520169406391599</v>
+      </c>
+      <c r="H3">
+        <v>0.55056005375619499</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="4">
-        <v>6.9729490089999997</v>
-      </c>
-      <c r="C4" s="4">
-        <v>6.9738571880000002</v>
-      </c>
-      <c r="D4" s="4">
-        <v>6.9651783140000001</v>
+      <c r="B4">
+        <v>4.70931514688424</v>
+      </c>
+      <c r="C4">
+        <v>1.89002910510055</v>
+      </c>
+      <c r="D4">
+        <v>1.6364320804784001</v>
+      </c>
+      <c r="E4">
+        <v>1.45456229910751</v>
+      </c>
+      <c r="F4">
+        <v>2.6499463840000002</v>
+      </c>
+      <c r="G4">
+        <v>2.2937069970340298</v>
+      </c>
+      <c r="H4">
+        <v>2.13261506819175</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4">
-        <v>6.53033866</v>
-      </c>
-      <c r="C5" s="4">
-        <v>6.5313767699999996</v>
-      </c>
-      <c r="D5" s="4">
-        <v>6.5110522409999998</v>
+      <c r="B5">
+        <v>9.3909205349798395</v>
+      </c>
+      <c r="C5">
+        <v>5.8561611945997702</v>
+      </c>
+      <c r="D5">
+        <v>5.31695784908832</v>
+      </c>
+      <c r="E5">
+        <v>4.88857483724105</v>
+      </c>
+      <c r="F5">
+        <v>7.154769494</v>
+      </c>
+      <c r="G5">
+        <v>6.5969477717673701</v>
+      </c>
+      <c r="H5">
+        <v>6.3168236910215301</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>4.4203874392245099</v>
+      </c>
+      <c r="C6">
+        <v>4.4381703570595796</v>
+      </c>
+      <c r="D6">
+        <v>4.43961470353669</v>
+      </c>
+      <c r="E6">
+        <v>4.4406803791778398</v>
+      </c>
+      <c r="F6">
+        <v>4.4336164349900598</v>
+      </c>
+      <c r="G6">
+        <v>4.4357324774038096</v>
+      </c>
+      <c r="H6">
+        <v>4.4367143228592703</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>7</v>
-      </c>
-      <c r="B6" s="4">
-        <v>7.986455479</v>
-      </c>
-      <c r="C6" s="4">
-        <v>7.9871286640000001</v>
-      </c>
-      <c r="D6" s="4">
-        <v>8.0195223710000008</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>0</v>
       </c>
       <c r="B9" t="s">
         <v>1</v>
@@ -4539,376 +4878,451 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" t="s">
         <v>3</v>
       </c>
+      <c r="F9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="4">
-        <v>18.421462741213698</v>
-      </c>
-      <c r="C10" s="4">
-        <v>18.416951952933001</v>
-      </c>
-      <c r="D10" s="4">
-        <v>18.475893918431499</v>
+      <c r="B10" s="2">
+        <f t="shared" ref="B10:E13" si="0">ABS((C3-$B3)/$B3)</f>
+        <v>0.65130671037862298</v>
+      </c>
+      <c r="C10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.70001002347703545</v>
+      </c>
+      <c r="D10" s="2">
+        <f>ABS((E3-$B3)/$B3)</f>
+        <v>0.73440969512298893</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.49875702575774439</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" ref="F10:G13" si="1">ABS((G3-$B3)/$B3)</f>
+        <v>0.57166212151054641</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="1"/>
+        <v>0.60378855141221444</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="4">
-        <v>17.266254811593701</v>
-      </c>
-      <c r="C11" s="4">
-        <v>17.267316870122901</v>
-      </c>
-      <c r="D11" s="4">
-        <v>17.345315007912301</v>
+      <c r="B11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.59866157898754679</v>
+      </c>
+      <c r="C11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.65251166476699052</v>
+      </c>
+      <c r="D11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.69113082184150021</v>
+      </c>
+      <c r="E11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.4372968677296426</v>
+      </c>
+      <c r="F11" s="2">
+        <f t="shared" si="1"/>
+        <v>0.51294255629683572</v>
+      </c>
+      <c r="G11" s="2">
+        <f t="shared" si="1"/>
+        <v>0.54714963817982687</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="4">
-        <v>17.154739436798899</v>
-      </c>
-      <c r="C12" s="4">
-        <v>17.157242310400498</v>
-      </c>
-      <c r="D12" s="4">
-        <v>17.237104830960799</v>
+      <c r="B12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.37640179439423377</v>
+      </c>
+      <c r="C12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.43381931203832358</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.47943603408933066</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.23811840731166831</v>
+      </c>
+      <c r="F12" s="2">
+        <f t="shared" si="1"/>
+        <v>0.29751851831833942</v>
+      </c>
+      <c r="G12" s="2">
+        <f t="shared" si="1"/>
+        <v>0.32734776452507902</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="4">
-        <v>17.596416562498199</v>
-      </c>
-      <c r="C13" s="4">
-        <v>17.5947611027206</v>
-      </c>
-      <c r="D13" s="4">
-        <v>17.667195454988001</v>
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <f t="shared" si="0"/>
+        <v>4.0229319442165084E-3</v>
+      </c>
+      <c r="C13" s="2">
+        <f t="shared" si="0"/>
+        <v>4.3496785240058414E-3</v>
+      </c>
+      <c r="D13" s="2">
+        <f t="shared" si="0"/>
+        <v>4.5907604779751848E-3</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="0"/>
+        <v>2.9927231373797041E-3</v>
+      </c>
+      <c r="F13" s="2">
+        <f t="shared" si="1"/>
+        <v>3.4714238039712914E-3</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" si="1"/>
+        <v>3.6935413149270504E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" t="s">
         <v>14</v>
       </c>
+      <c r="G19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" t="s">
+        <v>14</v>
+      </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" t="s">
-        <v>7</v>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20">
+        <v>9.8244659297066494</v>
+      </c>
+      <c r="C20">
+        <v>9.7224180529970603</v>
+      </c>
+      <c r="D20">
+        <v>9.7234960825768297</v>
+      </c>
+      <c r="F20" t="s">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>18.999836109635002</v>
+      </c>
+      <c r="H20">
+        <v>18.960935417712399</v>
+      </c>
+      <c r="I20">
+        <v>18.953478159908499</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21">
+        <v>7.1216328725202001</v>
+      </c>
+      <c r="C21">
+        <v>7.1373449227254699</v>
+      </c>
+      <c r="D21">
+        <v>7.13992117567118</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>17.9942031022752</v>
+      </c>
+      <c r="H21">
+        <v>17.929346810569498</v>
+      </c>
+      <c r="I21">
+        <v>17.933775911685199</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22">
+        <v>6.6593933989619503</v>
+      </c>
+      <c r="C22">
+        <v>6.6838920896256004</v>
+      </c>
+      <c r="D22">
+        <v>6.6868031512495696</v>
+      </c>
+      <c r="F22" t="s">
+        <v>2</v>
+      </c>
+      <c r="G22">
+        <v>17.898851255607799</v>
+      </c>
+      <c r="H22">
+        <v>17.829620432322201</v>
+      </c>
+      <c r="I22">
+        <v>17.837091601035802</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23">
+        <v>6.2782669680430798</v>
+      </c>
+      <c r="C23">
+        <v>6.3077024160821704</v>
+      </c>
+      <c r="D23">
+        <v>6.3109014900087397</v>
+      </c>
+      <c r="F23" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23">
+        <v>17.828724632559101</v>
+      </c>
+      <c r="H23">
+        <v>17.755691809499801</v>
+      </c>
+      <c r="I23">
+        <v>17.765996232382701</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24">
+        <v>8.17196340201785</v>
+      </c>
+      <c r="C24">
+        <v>8.1558525860663007</v>
+      </c>
+      <c r="D24">
+        <v>8.1577491532673392</v>
+      </c>
+      <c r="F24" t="s">
+        <v>3</v>
+      </c>
+      <c r="G24">
+        <v>18.273403916763399</v>
+      </c>
+      <c r="H24">
+        <v>18.218137121061599</v>
+      </c>
+      <c r="I24">
+        <v>18.216916221474101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="1">
-        <f>ABS((C4-C3)/C3)</f>
-        <v>0.26813971054574604</v>
-      </c>
-      <c r="C18" s="1">
-        <f>ABS((C5-C3)/C3)</f>
-        <v>0.31457511036330243</v>
-      </c>
-      <c r="D18" s="1">
-        <f>ABS((C6-C3)/C3)</f>
-        <v>0.16180355600029117</v>
+      <c r="B25">
+        <v>7.7303847693785599</v>
+      </c>
+      <c r="C25">
+        <v>7.7296829173204999</v>
+      </c>
+      <c r="D25">
+        <v>7.7318502195569998</v>
+      </c>
+      <c r="F25" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25">
+        <v>18.144490048353099</v>
+      </c>
+      <c r="H25">
+        <v>18.085211123354199</v>
+      </c>
+      <c r="I25">
+        <v>18.086176589070998</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="1">
-        <f>ABS((C11-C10)/C10)</f>
-        <v>6.2422657438003161E-2</v>
-      </c>
-      <c r="C19" s="1">
-        <f>ABS((C12-C10)/C10)</f>
-        <v>6.8399464023789616E-2</v>
-      </c>
-      <c r="D19" s="1">
-        <f>ABS((C13-C10)/C10)</f>
-        <v>4.4643155518547271E-2</v>
+      <c r="B26">
+        <v>7.5034105576629297</v>
+      </c>
+      <c r="C26">
+        <v>7.5094799929563196</v>
+      </c>
+      <c r="D26">
+        <v>7.5117951079559404</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26">
+        <v>18.0848329565383</v>
+      </c>
+      <c r="H26">
+        <v>18.023485724756899</v>
+      </c>
+      <c r="I26">
+        <v>18.025678930195902</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2</v>
+      </c>
+      <c r="D29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" t="s">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="2"/>
+      <c r="B30" s="2">
+        <f>ABS((D21-D20)/D20)</f>
+        <v>0.26570431920418636</v>
+      </c>
+      <c r="C30" s="2">
+        <f>ABS((D22-D20)/D20)</f>
+        <v>0.31230463873673964</v>
+      </c>
+      <c r="D30" s="2">
+        <f>ABS((D23-D20)/D20)</f>
+        <v>0.35096374427331656</v>
+      </c>
+      <c r="E30" s="2">
+        <f>ABS((D24-D20)/D20)</f>
+        <v>0.16102715690039657</v>
+      </c>
+      <c r="F30" s="2">
+        <f>ABS((D25-D20)/D20)</f>
+        <v>0.20482816531274034</v>
+      </c>
+      <c r="G30" s="2">
+        <f>ABS((D26-D20)/D20)</f>
+        <v>0.22745944008595365</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="2">
+        <f>ABS((I21-I20)/I20)</f>
+        <v>5.3800270305016301E-2</v>
+      </c>
+      <c r="C31" s="2">
+        <f>ABS((I22-I20)/I20)</f>
+        <v>5.8901408462017468E-2</v>
+      </c>
+      <c r="D31" s="2">
+        <f>ABS((I23-I20)/I20)</f>
+        <v>6.2652454473376251E-2</v>
+      </c>
+      <c r="E31" s="2">
+        <f>ABS((I24-I20)/I20)</f>
+        <v>3.8861571064693408E-2</v>
+      </c>
+      <c r="F31" s="2">
+        <f>ABS((I25-I20)/I20)</f>
+        <v>4.5759494036934495E-2</v>
+      </c>
+      <c r="G31" s="2">
+        <f>ABS((I26-I20)/I20)</f>
+        <v>4.8951396777143129E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-  <tableParts count="3">
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
-    <tablePart r:id="rId4"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC947F8-C987-4940-9A4B-AF550FDBA414}">
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" customWidth="1"/>
-    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="3">
-        <v>1.3491828990000001</v>
-      </c>
-      <c r="C3" s="3">
-        <v>0.47367235699999999</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0.40781563900000001</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0.68377695299999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3">
-        <v>4.5914016670000004</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1.848991979</v>
-      </c>
-      <c r="D4" s="3">
-        <v>1.6018056789999999</v>
-      </c>
-      <c r="E4" s="3">
-        <v>2.6036390140000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3">
-        <v>7.0140517329999996</v>
-      </c>
-      <c r="C5" s="3">
-        <v>3.45726975</v>
-      </c>
-      <c r="D5" s="3">
-        <v>3.0412965669999998</v>
-      </c>
-      <c r="E5" s="3">
-        <v>4.6174345839999997</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="3">
-        <v>9.2493070320000008</v>
-      </c>
-      <c r="C6" s="3">
-        <v>5.7607147589999999</v>
-      </c>
-      <c r="D6" s="3">
-        <v>5.229179222</v>
-      </c>
-      <c r="E6" s="3">
-        <v>7.0634611239999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="3">
-        <v>4.3528580320000003</v>
-      </c>
-      <c r="C7" s="3">
-        <v>4.3642715169999997</v>
-      </c>
-      <c r="D7" s="3">
-        <v>4.3652269190000004</v>
-      </c>
-      <c r="E7" s="3">
-        <v>4.361258791</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="1">
-        <f>ABS((C3-B3)/B3)</f>
-        <v>0.64891909217713861</v>
-      </c>
-      <c r="C12" s="1">
-        <f>ABS((D3-B3)/B3)</f>
-        <v>0.69773139038282461</v>
-      </c>
-      <c r="D12" s="1">
-        <f>ABS((E3-B3)/B3)</f>
-        <v>0.49319180260377737</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="1">
-        <f>ABS((C4-B4)/B4)</f>
-        <v>0.59729247992190537</v>
-      </c>
-      <c r="C13" s="1">
-        <f>ABS((D4-B4)/B4)</f>
-        <v>0.65112926396469861</v>
-      </c>
-      <c r="D13" s="1">
-        <f>ABS((E4-B4)/B4)</f>
-        <v>0.43293155275147049</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="1">
-        <f>ABS((C5-B5)/B5)</f>
-        <v>0.50709377666348043</v>
-      </c>
-      <c r="C14" s="1">
-        <f>ABS((D5-B5)/B5)</f>
-        <v>0.56639946741607528</v>
-      </c>
-      <c r="D14" s="1">
-        <f>ABS((E5-B5)/B5)</f>
-        <v>0.34168797725347488</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="1">
-        <f>ABS((C6-B6)/B6)</f>
-        <v>0.37717336671065765</v>
-      </c>
-      <c r="C15" s="1">
-        <f>ABS((D6-B6)/B6)</f>
-        <v>0.43464097322010065</v>
-      </c>
-      <c r="D15" s="1">
-        <f>ABS((E6-B6)/B6)</f>
-        <v>0.23632537015341679</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>18</v>
-      </c>
-      <c r="B16" s="1">
-        <f>ABS((C7-B7)/B7)</f>
-        <v>2.6220669077863896E-3</v>
-      </c>
-      <c r="C16" s="1">
-        <f>ABS((D7-B7)/B7)</f>
-        <v>2.8415553434250045E-3</v>
-      </c>
-      <c r="D16" s="1">
-        <f>ABS((E7-B7)/B7)</f>
-        <v>1.9299409579273184E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <tableParts count="2">
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>